<commit_message>
fixed failed tests, created new tests, refactored steps
</commit_message>
<xml_diff>
--- a/src/main/resources/Permanent Records.xlsx
+++ b/src/main/resources/Permanent Records.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE7C0BF-327C-4A4D-BF29-4D879506DB73}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3C04E1-57DB-4B44-8E94-8DEB4FBECDEB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="98">
   <si>
     <t>SAN DIEGO ELECTRICAL TRAINING TRUST</t>
   </si>
@@ -306,6 +306,24 @@
   </si>
   <si>
     <t xml:space="preserve">Every time use the same internal and external email addreses while creating users after every refresh  inorder to get email notifications </t>
+  </si>
+  <si>
+    <t>Automation Announcement for DueDateValidation</t>
+  </si>
+  <si>
+    <t>Automation Announcement for Application Intake and PreApplication</t>
+  </si>
+  <si>
+    <t>Automation Pre-App Announcement</t>
+  </si>
+  <si>
+    <t>All setting as Yes while announcement creation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> KPI and Focus Area = Yes ( other settings as NO)</t>
+  </si>
+  <si>
+    <t>Create  Announcement Type = Formula,with application due date with todays date ( to validate passed due date and closed oppuutunity)</t>
   </si>
 </sst>
 </file>
@@ -747,6 +765,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -779,9 +800,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1097,7 +1115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF2024B-3855-4F21-818F-72BDEF018EB6}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.44140625" customWidth="1"/>
@@ -1138,7 +1156,7 @@
       <c r="D4" s="16"/>
     </row>
     <row r="5" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="44" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1150,8 +1168,8 @@
       <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="32"/>
-      <c r="B6" s="41" t="s">
+      <c r="A6" s="35"/>
+      <c r="B6" s="44" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="12" t="s">
@@ -1160,16 +1178,16 @@
       <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="32"/>
-      <c r="B7" s="33"/>
+      <c r="A7" s="35"/>
+      <c r="B7" s="36"/>
       <c r="C7" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="16"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="32"/>
-      <c r="B8" s="38" t="s">
+      <c r="A8" s="35"/>
+      <c r="B8" s="41" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="12" t="s">
@@ -1178,15 +1196,15 @@
       <c r="D8" s="16"/>
     </row>
     <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="32"/>
-      <c r="B9" s="37"/>
+      <c r="A9" s="35"/>
+      <c r="B9" s="40"/>
       <c r="C9" s="11" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="16"/>
     </row>
     <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="32"/>
+      <c r="A10" s="35"/>
       <c r="B10" s="3" t="s">
         <v>13</v>
       </c>
@@ -1198,30 +1216,30 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="32"/>
-      <c r="B11" s="34" t="s">
+      <c r="A11" s="35"/>
+      <c r="B11" s="37" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="42" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="33"/>
-      <c r="B12" s="42"/>
+      <c r="A12" s="36"/>
+      <c r="B12" s="45"/>
       <c r="C12" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="40"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="31" t="s">
+      <c r="D12" s="43"/>
+    </row>
+    <row r="13" spans="1:4" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="37" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="12" t="s">
@@ -1231,9 +1249,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
-      <c r="B14" s="35"/>
+    <row r="14" spans="1:4" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="35"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="12" t="s">
         <v>20</v>
       </c>
@@ -1242,8 +1260,8 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="32"/>
-      <c r="B15" s="36"/>
+      <c r="A15" s="35"/>
+      <c r="B15" s="39"/>
       <c r="C15" s="30" t="s">
         <v>21</v>
       </c>
@@ -1251,257 +1269,249 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="33"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="11" t="s">
+    <row r="16" spans="1:4" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="35"/>
+      <c r="B16" s="39"/>
+      <c r="C16" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="35"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="35"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="34.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="36"/>
+      <c r="B19" s="40"/>
+      <c r="C19" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D19" s="16" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
+    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="11" t="s">
+      <c r="B20" s="5"/>
+      <c r="C20" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D20" s="16" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="31" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="38"/>
-      <c r="C18" s="12" t="s">
+      <c r="B21" s="41"/>
+      <c r="C21" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D21" s="16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="32"/>
-      <c r="B19" s="35"/>
-      <c r="C19" s="12" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="35"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D22" s="16" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="33"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="13" t="s">
+    <row r="23" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="36"/>
+      <c r="B23" s="40"/>
+      <c r="C23" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D23" s="16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C24" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D24" s="16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="21" t="s">
+    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="21" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B28" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="25" t="s">
+      <c r="C28" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="27" t="s">
+      <c r="D28" s="27" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="19" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B29" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C26" s="24" t="s">
+      <c r="C29" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D29" s="14" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="19" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="20" t="s">
+      <c r="B30" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C30" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="D30" s="14" t="s">
         <v>68</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="19" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C28" s="26"/>
-      <c r="D28" s="14" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="B29" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B30" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="C30" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" s="26"/>
+      <c r="D31" s="14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B31" s="20" t="s">
+      <c r="B34" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="C31" s="26" t="s">
+      <c r="C34" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="D34" s="14" t="s">
         <v>73</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="43" t="s">
+    <row r="41" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="31" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="45" t="s">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="B40" s="45" t="s">
+      <c r="B43" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="C40" s="45" t="s">
+      <c r="C43" s="33" t="s">
         <v>89</v>
-      </c>
-      <c r="D40" s="29"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B41" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="C41" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="D41" s="29"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B42" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C42" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="D42" s="29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B43" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="C43" s="20" t="s">
-        <v>85</v>
       </c>
       <c r="D43" s="29"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="14" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C44" s="20" t="s">
         <v>85</v>
@@ -1510,32 +1520,70 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="C45" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="D45" s="29"/>
+      <c r="D45" s="29" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="44" t="s">
+      <c r="A46" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B46" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C46" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D46" s="29"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D47" s="29"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D48" s="29"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="32" t="s">
         <v>86</v>
       </c>
-      <c r="B46" s="14"/>
-      <c r="C46" s="20" t="s">
+      <c r="B49" s="14"/>
+      <c r="C49" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D46" s="29"/>
+      <c r="D49" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="B13:B16"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="A13:A19"/>
+    <mergeCell ref="B13:B19"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
     <mergeCell ref="D11:D12"/>
     <mergeCell ref="A5:A12"/>
     <mergeCell ref="B6:B7"/>
@@ -1544,25 +1592,25 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D13" r:id="rId1" display="https://test8-internal--automation--c.visualforce.com/apex/AnnouncementView?id=a1b18000000t6fkAAA&amp;RefreshBehaviour=null&amp;TableName=ActiveFundingOpportunitiesAll&amp;TableType=flextable&amp;retURL=%2Fapex%2Fc__PhaseView%3Ft%3DFundingOpportunity" xr:uid="{C9FEE6D1-22A8-4E9E-8E5E-5AD9ED3718F8}"/>
-    <hyperlink ref="B41" r:id="rId2" xr:uid="{AF5F6C36-4969-4497-8391-22B2E0F63737}"/>
-    <hyperlink ref="B27" r:id="rId3" xr:uid="{49BE5B1F-DB58-465B-8C07-B50636BB4D9C}"/>
-    <hyperlink ref="B28" r:id="rId4" xr:uid="{67CC90BD-C434-48C4-B5A7-ADE1CBB64E55}"/>
-    <hyperlink ref="B29" r:id="rId5" xr:uid="{609E544F-B176-48AE-ADF1-696201254949}"/>
-    <hyperlink ref="B30" r:id="rId6" xr:uid="{3B4827AF-F449-4362-BDEB-A0F39720646E}"/>
-    <hyperlink ref="B31" r:id="rId7" xr:uid="{772F7E1F-4BF9-4DFB-BB1F-72E81C82B5C2}"/>
-    <hyperlink ref="C30" r:id="rId8" display="https://test8-internal--automation.my.salesforce.com/00E4T000000klGw" xr:uid="{F01024FA-1968-4218-96D8-5A1889369883}"/>
-    <hyperlink ref="C29" r:id="rId9" display="https://test8-internal--automation.my.salesforce.com/00E4T000000klGw" xr:uid="{F7DB9398-81F8-4ABB-B445-88CB49B5E29B}"/>
-    <hyperlink ref="B45" r:id="rId10" xr:uid="{A26EF93C-4FE6-4A75-BE85-63A3BDE6CBDB}"/>
-    <hyperlink ref="B26" r:id="rId11" xr:uid="{02E624E7-AE71-46E1-B1C9-A8B69F15DEAC}"/>
-    <hyperlink ref="B44" r:id="rId12" xr:uid="{928C4190-80E4-4614-8A9D-22EBA6EDDDC1}"/>
-    <hyperlink ref="B43" r:id="rId13" xr:uid="{A3D11415-D129-4A87-93F5-4E4B333B4DFB}"/>
-    <hyperlink ref="B42" r:id="rId14" xr:uid="{8942867D-7565-47B7-8A27-34B849A94365}"/>
-    <hyperlink ref="C46" r:id="rId15" display="mailto:external.user.product@gmail.com" xr:uid="{582FB88F-E237-4D3B-8C4A-763751EEF0EC}"/>
-    <hyperlink ref="C42" r:id="rId16" display="mailto:internal.user.product@gmail.com" xr:uid="{B0E25D6B-41F6-4A0C-AEBE-0E17B8D87033}"/>
-    <hyperlink ref="C43" r:id="rId17" display="mailto:internal.user.product@gmail.com" xr:uid="{0D31973E-8ABF-4D5E-9FD3-AB2031F2F8A2}"/>
-    <hyperlink ref="C44" r:id="rId18" display="mailto:internal.user.product@gmail.com" xr:uid="{D69E89E3-2B24-449B-AC15-4477AE77C01E}"/>
-    <hyperlink ref="C41" r:id="rId19" display="mailto:internal.user.product@gmail.com" xr:uid="{54B626CC-59F9-40AB-AC34-4DF492A7A583}"/>
-    <hyperlink ref="C45" r:id="rId20" display="mailto:internal.user.product@gmail.com" xr:uid="{06039687-AF31-4D97-84D3-62BD6A32505B}"/>
+    <hyperlink ref="B44" r:id="rId2" xr:uid="{AF5F6C36-4969-4497-8391-22B2E0F63737}"/>
+    <hyperlink ref="B30" r:id="rId3" xr:uid="{49BE5B1F-DB58-465B-8C07-B50636BB4D9C}"/>
+    <hyperlink ref="B31" r:id="rId4" xr:uid="{67CC90BD-C434-48C4-B5A7-ADE1CBB64E55}"/>
+    <hyperlink ref="B32" r:id="rId5" xr:uid="{609E544F-B176-48AE-ADF1-696201254949}"/>
+    <hyperlink ref="B33" r:id="rId6" xr:uid="{3B4827AF-F449-4362-BDEB-A0F39720646E}"/>
+    <hyperlink ref="B34" r:id="rId7" xr:uid="{772F7E1F-4BF9-4DFB-BB1F-72E81C82B5C2}"/>
+    <hyperlink ref="C33" r:id="rId8" display="https://test8-internal--automation.my.salesforce.com/00E4T000000klGw" xr:uid="{F01024FA-1968-4218-96D8-5A1889369883}"/>
+    <hyperlink ref="C32" r:id="rId9" display="https://test8-internal--automation.my.salesforce.com/00E4T000000klGw" xr:uid="{F7DB9398-81F8-4ABB-B445-88CB49B5E29B}"/>
+    <hyperlink ref="B48" r:id="rId10" xr:uid="{A26EF93C-4FE6-4A75-BE85-63A3BDE6CBDB}"/>
+    <hyperlink ref="B29" r:id="rId11" xr:uid="{02E624E7-AE71-46E1-B1C9-A8B69F15DEAC}"/>
+    <hyperlink ref="B47" r:id="rId12" xr:uid="{928C4190-80E4-4614-8A9D-22EBA6EDDDC1}"/>
+    <hyperlink ref="B46" r:id="rId13" xr:uid="{A3D11415-D129-4A87-93F5-4E4B333B4DFB}"/>
+    <hyperlink ref="B45" r:id="rId14" xr:uid="{8942867D-7565-47B7-8A27-34B849A94365}"/>
+    <hyperlink ref="C49" r:id="rId15" display="mailto:external.user.product@gmail.com" xr:uid="{582FB88F-E237-4D3B-8C4A-763751EEF0EC}"/>
+    <hyperlink ref="C45" r:id="rId16" display="mailto:internal.user.product@gmail.com" xr:uid="{B0E25D6B-41F6-4A0C-AEBE-0E17B8D87033}"/>
+    <hyperlink ref="C46" r:id="rId17" display="mailto:internal.user.product@gmail.com" xr:uid="{0D31973E-8ABF-4D5E-9FD3-AB2031F2F8A2}"/>
+    <hyperlink ref="C47" r:id="rId18" display="mailto:internal.user.product@gmail.com" xr:uid="{D69E89E3-2B24-449B-AC15-4477AE77C01E}"/>
+    <hyperlink ref="C44" r:id="rId19" display="mailto:internal.user.product@gmail.com" xr:uid="{54B626CC-59F9-40AB-AC34-4DF492A7A583}"/>
+    <hyperlink ref="C48" r:id="rId20" display="mailto:internal.user.product@gmail.com" xr:uid="{06039687-AF31-4D97-84D3-62BD6A32505B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId21"/>

</xml_diff>